<commit_message>
ci(dev): publish dev build from bb67177da9562b73a463f0e76b978c1a873e03db bb67177da9562b73a463f0e76b978c1a873e03db
</commit_message>
<xml_diff>
--- a/dev/StructureDefinition-ph-core-practitionerrole.xlsx
+++ b/dev/StructureDefinition-ph-core-practitionerrole.xlsx
@@ -10,13 +10,13 @@
     <sheet name="Elements" r:id="rId4" sheetId="2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AN$43</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AN$54</definedName>
   </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1579" uniqueCount="325">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1977" uniqueCount="383">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-03-25T03:48:45+00:00</t>
+    <t>2026-03-25T03:54:03+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -621,6 +621,213 @@
     <t>.code</t>
   </si>
   <si>
+    <t>PractitionerRole.code.id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">string
+</t>
+  </si>
+  <si>
+    <t>Unique id for inter-element referencing</t>
+  </si>
+  <si>
+    <t>Unique id for the element within a resource (for internal references). This may be any string value that does not contain spaces.</t>
+  </si>
+  <si>
+    <t>Element.id</t>
+  </si>
+  <si>
+    <t>n/a</t>
+  </si>
+  <si>
+    <t>PractitionerRole.code.extension</t>
+  </si>
+  <si>
+    <t>May be used to represent additional information that is not part of the basic definition of the element. To make the use of extensions safe and manageable, there is a strict set of governance  applied to the definition and use of extensions. Though any implementer can define an extension, there is a set of requirements that SHALL be met as part of the definition of the extension.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">value:url}
+</t>
+  </si>
+  <si>
+    <t>Extensions are always sliced by (at least) url</t>
+  </si>
+  <si>
+    <t>open</t>
+  </si>
+  <si>
+    <t>Element.extension</t>
+  </si>
+  <si>
+    <t>PractitionerRole.code.coding</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coding
+</t>
+  </si>
+  <si>
+    <t>Code defined by a terminology system</t>
+  </si>
+  <si>
+    <t>A reference to a code defined by a terminology system.</t>
+  </si>
+  <si>
+    <t>Codes may be defined very casually in enumerations, or code lists, up to very formal definitions such as SNOMED CT - see the HL7 v3 Core Principles for more information.  Ordering of codings is undefined and SHALL NOT be used to infer meaning. Generally, at most only one of the coding values will be labeled as UserSelected = true.</t>
+  </si>
+  <si>
+    <t>Allows for alternative encodings within a code system, and translations to other code systems.</t>
+  </si>
+  <si>
+    <t>CodeableConcept.coding</t>
+  </si>
+  <si>
+    <t>C*E.1-8, C*E.10-22</t>
+  </si>
+  <si>
+    <t>union(., ./translation)</t>
+  </si>
+  <si>
+    <t>PractitionerRole.code.coding.id</t>
+  </si>
+  <si>
+    <t>PractitionerRole.code.coding.extension</t>
+  </si>
+  <si>
+    <t>PractitionerRole.code.coding.system</t>
+  </si>
+  <si>
+    <t>Identity of the terminology system</t>
+  </si>
+  <si>
+    <t>The identification of the code system that defines the meaning of the symbol in the code.</t>
+  </si>
+  <si>
+    <t>The URI may be an OID (urn:oid:...) or a UUID (urn:uuid:...).  OIDs and UUIDs SHALL be references to the HL7 OID registry. Otherwise, the URI should come from HL7's list of FHIR defined special URIs or it should reference to some definition that establishes the system clearly and unambiguously.</t>
+  </si>
+  <si>
+    <t>Need to be unambiguous about the source of the definition of the symbol.</t>
+  </si>
+  <si>
+    <t>Coding.system</t>
+  </si>
+  <si>
+    <t>C*E.3</t>
+  </si>
+  <si>
+    <t>./codeSystem</t>
+  </si>
+  <si>
+    <t>PractitionerRole.code.coding.version</t>
+  </si>
+  <si>
+    <t>Version of the system - if relevant</t>
+  </si>
+  <si>
+    <t>The version of the code system which was used when choosing this code. Note that a well-maintained code system does not need the version reported, because the meaning of codes is consistent across versions. However this cannot consistently be assured, and when the meaning is not guaranteed to be consistent, the version SHOULD be exchanged.</t>
+  </si>
+  <si>
+    <t>Where the terminology does not clearly define what string should be used to identify code system versions, the recommendation is to use the date (expressed in FHIR date format) on which that version was officially published as the version date.</t>
+  </si>
+  <si>
+    <t>Coding.version</t>
+  </si>
+  <si>
+    <t>C*E.7</t>
+  </si>
+  <si>
+    <t>./codeSystemVersion</t>
+  </si>
+  <si>
+    <t>PractitionerRole.code.coding.code</t>
+  </si>
+  <si>
+    <t>Symbol in syntax defined by the system</t>
+  </si>
+  <si>
+    <t>A symbol in syntax defined by the system. The symbol may be a predefined code or an expression in a syntax defined by the coding system (e.g. post-coordination).</t>
+  </si>
+  <si>
+    <t>Need to refer to a particular code in the system.</t>
+  </si>
+  <si>
+    <t>Coding.code</t>
+  </si>
+  <si>
+    <t>C*E.1</t>
+  </si>
+  <si>
+    <t>./code</t>
+  </si>
+  <si>
+    <t>PractitionerRole.code.coding.display</t>
+  </si>
+  <si>
+    <t>Representation defined by the system</t>
+  </si>
+  <si>
+    <t>A representation of the meaning of the code in the system, following the rules of the system.</t>
+  </si>
+  <si>
+    <t>Need to be able to carry a human-readable meaning of the code for readers that do not know  the system.</t>
+  </si>
+  <si>
+    <t>Coding.display</t>
+  </si>
+  <si>
+    <t>C*E.2 - but note this is not well followed</t>
+  </si>
+  <si>
+    <t>CV.displayName</t>
+  </si>
+  <si>
+    <t>PractitionerRole.code.coding.userSelected</t>
+  </si>
+  <si>
+    <t>If this coding was chosen directly by the user</t>
+  </si>
+  <si>
+    <t>Indicates that this coding was chosen by a user directly - e.g. off a pick list of available items (codes or displays).</t>
+  </si>
+  <si>
+    <t>Amongst a set of alternatives, a directly chosen code is the most appropriate starting point for new translations. There is some ambiguity about what exactly 'directly chosen' implies, and trading partner agreement may be needed to clarify the use of this element and its consequences more completely.</t>
+  </si>
+  <si>
+    <t>This has been identified as a clinical safety criterium - that this exact system/code pair was chosen explicitly, rather than inferred by the system based on some rules or language processing.</t>
+  </si>
+  <si>
+    <t>Coding.userSelected</t>
+  </si>
+  <si>
+    <t>Sometimes implied by being first</t>
+  </si>
+  <si>
+    <t>CD.codingRationale</t>
+  </si>
+  <si>
+    <t>PractitionerRole.code.text</t>
+  </si>
+  <si>
+    <t>Plain text representation of the concept</t>
+  </si>
+  <si>
+    <t>A human language representation of the concept as seen/selected/uttered by the user who entered the data and/or which represents the intended meaning of the user.</t>
+  </si>
+  <si>
+    <t>Very often the text is the same as a displayName of one of the codings.</t>
+  </si>
+  <si>
+    <t>The codes from the terminologies do not always capture the correct meaning with all the nuances of the human using them, or sometimes there is no appropriate code at all. In these cases, the text is used to capture the full meaning of the source.</t>
+  </si>
+  <si>
+    <t>CodeableConcept.text</t>
+  </si>
+  <si>
+    <t>C*E.9. But note many systems use C*E.2 for this</t>
+  </si>
+  <si>
+    <t>./originalText[mediaType/code="text/plain"]/data</t>
+  </si>
+  <si>
     <t>PractitionerRole.specialty</t>
   </si>
   <si>
@@ -708,39 +915,7 @@
     <t>PractitionerRole.telecom.id</t>
   </si>
   <si>
-    <t xml:space="preserve">string
-</t>
-  </si>
-  <si>
-    <t>Unique id for inter-element referencing</t>
-  </si>
-  <si>
-    <t>Unique id for the element within a resource (for internal references). This may be any string value that does not contain spaces.</t>
-  </si>
-  <si>
-    <t>Element.id</t>
-  </si>
-  <si>
-    <t>n/a</t>
-  </si>
-  <si>
     <t>PractitionerRole.telecom.extension</t>
-  </si>
-  <si>
-    <t>May be used to represent additional information that is not part of the basic definition of the element. To make the use of extensions safe and manageable, there is a strict set of governance  applied to the definition and use of extensions. Though any implementer can define an extension, there is a set of requirements that SHALL be met as part of the definition of the extension.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">value:url}
-</t>
-  </si>
-  <si>
-    <t>Extensions are always sliced by (at least) url</t>
-  </si>
-  <si>
-    <t>open</t>
-  </si>
-  <si>
-    <t>Element.extension</t>
   </si>
   <si>
     <t>PractitionerRole.telecom.system</t>
@@ -1342,7 +1517,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AN43"/>
+  <dimension ref="A1:AN54"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="40.26953125" customWidth="true" bestFit="true"/>
@@ -3218,7 +3393,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" hidden="true">
       <c r="A17" t="s" s="2">
         <v>194</v>
       </c>
@@ -3234,25 +3409,25 @@
         <v>78</v>
       </c>
       <c r="G17" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="H17" t="s" s="2">
-        <v>89</v>
+        <v>77</v>
       </c>
       <c r="I17" t="s" s="2">
         <v>77</v>
       </c>
       <c r="J17" t="s" s="2">
-        <v>89</v>
+        <v>77</v>
       </c>
       <c r="K17" t="s" s="2">
-        <v>184</v>
+        <v>195</v>
       </c>
       <c r="L17" t="s" s="2">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="M17" t="s" s="2">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="N17" s="2"/>
       <c r="O17" s="2"/>
@@ -3279,52 +3454,52 @@
         <v>77</v>
       </c>
       <c r="X17" t="s" s="2">
-        <v>112</v>
+        <v>77</v>
       </c>
       <c r="Y17" t="s" s="2">
-        <v>197</v>
+        <v>77</v>
       </c>
       <c r="Z17" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AA17" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AB17" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AC17" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AD17" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AE17" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AF17" t="s" s="2">
         <v>198</v>
       </c>
-      <c r="AA17" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AB17" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AC17" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AD17" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AE17" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AF17" t="s" s="2">
-        <v>194</v>
-      </c>
       <c r="AG17" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH17" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="AI17" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AJ17" t="s" s="2">
-        <v>100</v>
+        <v>77</v>
       </c>
       <c r="AK17" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AL17" t="s" s="2">
         <v>199</v>
       </c>
-      <c r="AL17" t="s" s="2">
-        <v>200</v>
-      </c>
       <c r="AM17" t="s" s="2">
-        <v>201</v>
+        <v>77</v>
       </c>
       <c r="AN17" t="s" s="2">
         <v>77</v>
@@ -3332,14 +3507,14 @@
     </row>
     <row r="18" hidden="true">
       <c r="A18" t="s" s="2">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="B18" t="s" s="2">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" t="s" s="2">
-        <v>77</v>
+        <v>133</v>
       </c>
       <c r="E18" s="2"/>
       <c r="F18" t="s" s="2">
@@ -3355,18 +3530,20 @@
         <v>77</v>
       </c>
       <c r="J18" t="s" s="2">
-        <v>89</v>
+        <v>77</v>
       </c>
       <c r="K18" t="s" s="2">
-        <v>203</v>
+        <v>134</v>
       </c>
       <c r="L18" t="s" s="2">
-        <v>204</v>
+        <v>135</v>
       </c>
       <c r="M18" t="s" s="2">
-        <v>205</v>
-      </c>
-      <c r="N18" s="2"/>
+        <v>201</v>
+      </c>
+      <c r="N18" t="s" s="2">
+        <v>137</v>
+      </c>
       <c r="O18" s="2"/>
       <c r="P18" t="s" s="2">
         <v>77</v>
@@ -3403,19 +3580,19 @@
         <v>77</v>
       </c>
       <c r="AB18" t="s" s="2">
-        <v>77</v>
+        <v>202</v>
       </c>
       <c r="AC18" t="s" s="2">
-        <v>77</v>
+        <v>203</v>
       </c>
       <c r="AD18" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AE18" t="s" s="2">
-        <v>77</v>
+        <v>204</v>
       </c>
       <c r="AF18" t="s" s="2">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="AG18" t="s" s="2">
         <v>78</v>
@@ -3427,27 +3604,27 @@
         <v>77</v>
       </c>
       <c r="AJ18" t="s" s="2">
-        <v>100</v>
+        <v>139</v>
       </c>
       <c r="AK18" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AL18" t="s" s="2">
+        <v>199</v>
+      </c>
+      <c r="AM18" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AN18" t="s" s="2">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s" s="2">
         <v>206</v>
       </c>
-      <c r="AM18" t="s" s="2">
-        <v>207</v>
-      </c>
-      <c r="AN18" t="s" s="2">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="19" hidden="true">
-      <c r="A19" t="s" s="2">
-        <v>209</v>
-      </c>
       <c r="B19" t="s" s="2">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" t="s" s="2">
@@ -3461,25 +3638,29 @@
         <v>79</v>
       </c>
       <c r="H19" t="s" s="2">
-        <v>77</v>
+        <v>89</v>
       </c>
       <c r="I19" t="s" s="2">
         <v>77</v>
       </c>
       <c r="J19" t="s" s="2">
-        <v>77</v>
+        <v>89</v>
       </c>
       <c r="K19" t="s" s="2">
+        <v>207</v>
+      </c>
+      <c r="L19" t="s" s="2">
+        <v>208</v>
+      </c>
+      <c r="M19" t="s" s="2">
+        <v>209</v>
+      </c>
+      <c r="N19" t="s" s="2">
         <v>210</v>
       </c>
-      <c r="L19" t="s" s="2">
+      <c r="O19" t="s" s="2">
         <v>211</v>
       </c>
-      <c r="M19" t="s" s="2">
-        <v>212</v>
-      </c>
-      <c r="N19" s="2"/>
-      <c r="O19" s="2"/>
       <c r="P19" t="s" s="2">
         <v>77</v>
       </c>
@@ -3527,7 +3708,7 @@
         <v>77</v>
       </c>
       <c r="AF19" t="s" s="2">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="AG19" t="s" s="2">
         <v>78</v>
@@ -3554,7 +3735,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" hidden="true">
       <c r="A20" t="s" s="2">
         <v>215</v>
       </c>
@@ -3570,30 +3751,28 @@
         <v>78</v>
       </c>
       <c r="G20" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="H20" t="s" s="2">
-        <v>89</v>
+        <v>77</v>
       </c>
       <c r="I20" t="s" s="2">
         <v>77</v>
       </c>
       <c r="J20" t="s" s="2">
-        <v>89</v>
+        <v>77</v>
       </c>
       <c r="K20" t="s" s="2">
-        <v>216</v>
+        <v>195</v>
       </c>
       <c r="L20" t="s" s="2">
-        <v>217</v>
+        <v>196</v>
       </c>
       <c r="M20" t="s" s="2">
-        <v>218</v>
+        <v>197</v>
       </c>
       <c r="N20" s="2"/>
-      <c r="O20" t="s" s="2">
-        <v>219</v>
-      </c>
+      <c r="O20" s="2"/>
       <c r="P20" t="s" s="2">
         <v>77</v>
       </c>
@@ -3641,25 +3820,25 @@
         <v>77</v>
       </c>
       <c r="AF20" t="s" s="2">
-        <v>215</v>
+        <v>198</v>
       </c>
       <c r="AG20" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH20" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="AI20" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AJ20" t="s" s="2">
-        <v>100</v>
+        <v>77</v>
       </c>
       <c r="AK20" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AL20" t="s" s="2">
-        <v>220</v>
+        <v>199</v>
       </c>
       <c r="AM20" t="s" s="2">
         <v>77</v>
@@ -3670,21 +3849,21 @@
     </row>
     <row r="21" hidden="true">
       <c r="A21" t="s" s="2">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="B21" t="s" s="2">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21" t="s" s="2">
-        <v>77</v>
+        <v>133</v>
       </c>
       <c r="E21" s="2"/>
       <c r="F21" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G21" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="H21" t="s" s="2">
         <v>77</v>
@@ -3696,15 +3875,17 @@
         <v>77</v>
       </c>
       <c r="K21" t="s" s="2">
-        <v>222</v>
+        <v>134</v>
       </c>
       <c r="L21" t="s" s="2">
-        <v>223</v>
+        <v>135</v>
       </c>
       <c r="M21" t="s" s="2">
-        <v>224</v>
-      </c>
-      <c r="N21" s="2"/>
+        <v>201</v>
+      </c>
+      <c r="N21" t="s" s="2">
+        <v>137</v>
+      </c>
       <c r="O21" s="2"/>
       <c r="P21" t="s" s="2">
         <v>77</v>
@@ -3741,37 +3922,37 @@
         <v>77</v>
       </c>
       <c r="AB21" t="s" s="2">
-        <v>77</v>
+        <v>202</v>
       </c>
       <c r="AC21" t="s" s="2">
-        <v>77</v>
+        <v>203</v>
       </c>
       <c r="AD21" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AE21" t="s" s="2">
-        <v>77</v>
+        <v>204</v>
       </c>
       <c r="AF21" t="s" s="2">
-        <v>225</v>
+        <v>205</v>
       </c>
       <c r="AG21" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH21" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="AI21" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AJ21" t="s" s="2">
-        <v>77</v>
+        <v>139</v>
       </c>
       <c r="AK21" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AL21" t="s" s="2">
-        <v>226</v>
+        <v>199</v>
       </c>
       <c r="AM21" t="s" s="2">
         <v>77</v>
@@ -3782,21 +3963,21 @@
     </row>
     <row r="22" hidden="true">
       <c r="A22" t="s" s="2">
-        <v>227</v>
+        <v>217</v>
       </c>
       <c r="B22" t="s" s="2">
-        <v>227</v>
+        <v>217</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" t="s" s="2">
-        <v>133</v>
+        <v>77</v>
       </c>
       <c r="E22" s="2"/>
       <c r="F22" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G22" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="H22" t="s" s="2">
         <v>77</v>
@@ -3805,21 +3986,23 @@
         <v>77</v>
       </c>
       <c r="J22" t="s" s="2">
-        <v>77</v>
+        <v>89</v>
       </c>
       <c r="K22" t="s" s="2">
-        <v>134</v>
+        <v>102</v>
       </c>
       <c r="L22" t="s" s="2">
-        <v>135</v>
+        <v>218</v>
       </c>
       <c r="M22" t="s" s="2">
-        <v>228</v>
+        <v>219</v>
       </c>
       <c r="N22" t="s" s="2">
-        <v>137</v>
-      </c>
-      <c r="O22" s="2"/>
+        <v>220</v>
+      </c>
+      <c r="O22" t="s" s="2">
+        <v>221</v>
+      </c>
       <c r="P22" t="s" s="2">
         <v>77</v>
       </c>
@@ -3855,37 +4038,37 @@
         <v>77</v>
       </c>
       <c r="AB22" t="s" s="2">
-        <v>229</v>
+        <v>77</v>
       </c>
       <c r="AC22" t="s" s="2">
-        <v>230</v>
+        <v>77</v>
       </c>
       <c r="AD22" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AE22" t="s" s="2">
-        <v>231</v>
+        <v>77</v>
       </c>
       <c r="AF22" t="s" s="2">
-        <v>232</v>
+        <v>222</v>
       </c>
       <c r="AG22" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH22" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="AI22" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AJ22" t="s" s="2">
-        <v>139</v>
+        <v>100</v>
       </c>
       <c r="AK22" t="s" s="2">
-        <v>77</v>
+        <v>223</v>
       </c>
       <c r="AL22" t="s" s="2">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="AM22" t="s" s="2">
         <v>77</v>
@@ -3894,12 +4077,12 @@
         <v>77</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" hidden="true">
       <c r="A23" t="s" s="2">
-        <v>233</v>
+        <v>225</v>
       </c>
       <c r="B23" t="s" s="2">
-        <v>233</v>
+        <v>225</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" t="s" s="2">
@@ -3913,7 +4096,7 @@
         <v>88</v>
       </c>
       <c r="H23" t="s" s="2">
-        <v>89</v>
+        <v>77</v>
       </c>
       <c r="I23" t="s" s="2">
         <v>77</v>
@@ -3922,15 +4105,17 @@
         <v>89</v>
       </c>
       <c r="K23" t="s" s="2">
-        <v>108</v>
+        <v>195</v>
       </c>
       <c r="L23" t="s" s="2">
-        <v>234</v>
+        <v>226</v>
       </c>
       <c r="M23" t="s" s="2">
-        <v>235</v>
-      </c>
-      <c r="N23" s="2"/>
+        <v>227</v>
+      </c>
+      <c r="N23" t="s" s="2">
+        <v>228</v>
+      </c>
       <c r="O23" s="2"/>
       <c r="P23" t="s" s="2">
         <v>77</v>
@@ -3955,13 +4140,13 @@
         <v>77</v>
       </c>
       <c r="X23" t="s" s="2">
-        <v>236</v>
+        <v>77</v>
       </c>
       <c r="Y23" t="s" s="2">
-        <v>237</v>
+        <v>77</v>
       </c>
       <c r="Z23" t="s" s="2">
-        <v>238</v>
+        <v>77</v>
       </c>
       <c r="AA23" t="s" s="2">
         <v>77</v>
@@ -3979,7 +4164,7 @@
         <v>77</v>
       </c>
       <c r="AF23" t="s" s="2">
-        <v>239</v>
+        <v>229</v>
       </c>
       <c r="AG23" t="s" s="2">
         <v>78</v>
@@ -3988,19 +4173,19 @@
         <v>88</v>
       </c>
       <c r="AI23" t="s" s="2">
-        <v>240</v>
+        <v>77</v>
       </c>
       <c r="AJ23" t="s" s="2">
         <v>100</v>
       </c>
       <c r="AK23" t="s" s="2">
-        <v>241</v>
+        <v>230</v>
       </c>
       <c r="AL23" t="s" s="2">
-        <v>242</v>
+        <v>231</v>
       </c>
       <c r="AM23" t="s" s="2">
-        <v>243</v>
+        <v>77</v>
       </c>
       <c r="AN23" t="s" s="2">
         <v>77</v>
@@ -4008,10 +4193,10 @@
     </row>
     <row r="24">
       <c r="A24" t="s" s="2">
-        <v>244</v>
+        <v>232</v>
       </c>
       <c r="B24" t="s" s="2">
-        <v>244</v>
+        <v>232</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" t="s" s="2">
@@ -4034,19 +4219,17 @@
         <v>89</v>
       </c>
       <c r="K24" t="s" s="2">
-        <v>222</v>
+        <v>108</v>
       </c>
       <c r="L24" t="s" s="2">
-        <v>245</v>
+        <v>233</v>
       </c>
       <c r="M24" t="s" s="2">
-        <v>246</v>
-      </c>
-      <c r="N24" t="s" s="2">
-        <v>247</v>
-      </c>
+        <v>234</v>
+      </c>
+      <c r="N24" s="2"/>
       <c r="O24" t="s" s="2">
-        <v>248</v>
+        <v>235</v>
       </c>
       <c r="P24" t="s" s="2">
         <v>77</v>
@@ -4095,7 +4278,7 @@
         <v>77</v>
       </c>
       <c r="AF24" t="s" s="2">
-        <v>249</v>
+        <v>236</v>
       </c>
       <c r="AG24" t="s" s="2">
         <v>78</v>
@@ -4110,13 +4293,13 @@
         <v>100</v>
       </c>
       <c r="AK24" t="s" s="2">
-        <v>250</v>
+        <v>237</v>
       </c>
       <c r="AL24" t="s" s="2">
-        <v>251</v>
+        <v>238</v>
       </c>
       <c r="AM24" t="s" s="2">
-        <v>252</v>
+        <v>77</v>
       </c>
       <c r="AN24" t="s" s="2">
         <v>77</v>
@@ -4124,10 +4307,10 @@
     </row>
     <row r="25" hidden="true">
       <c r="A25" t="s" s="2">
-        <v>253</v>
+        <v>239</v>
       </c>
       <c r="B25" t="s" s="2">
-        <v>253</v>
+        <v>239</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" t="s" s="2">
@@ -4144,25 +4327,23 @@
         <v>77</v>
       </c>
       <c r="I25" t="s" s="2">
-        <v>89</v>
+        <v>77</v>
       </c>
       <c r="J25" t="s" s="2">
         <v>89</v>
       </c>
       <c r="K25" t="s" s="2">
-        <v>108</v>
+        <v>195</v>
       </c>
       <c r="L25" t="s" s="2">
-        <v>254</v>
+        <v>240</v>
       </c>
       <c r="M25" t="s" s="2">
-        <v>255</v>
-      </c>
-      <c r="N25" t="s" s="2">
-        <v>256</v>
-      </c>
+        <v>241</v>
+      </c>
+      <c r="N25" s="2"/>
       <c r="O25" t="s" s="2">
-        <v>257</v>
+        <v>242</v>
       </c>
       <c r="P25" t="s" s="2">
         <v>77</v>
@@ -4187,13 +4368,13 @@
         <v>77</v>
       </c>
       <c r="X25" t="s" s="2">
-        <v>236</v>
+        <v>77</v>
       </c>
       <c r="Y25" t="s" s="2">
-        <v>258</v>
+        <v>77</v>
       </c>
       <c r="Z25" t="s" s="2">
-        <v>259</v>
+        <v>77</v>
       </c>
       <c r="AA25" t="s" s="2">
         <v>77</v>
@@ -4211,7 +4392,7 @@
         <v>77</v>
       </c>
       <c r="AF25" t="s" s="2">
-        <v>260</v>
+        <v>243</v>
       </c>
       <c r="AG25" t="s" s="2">
         <v>78</v>
@@ -4226,13 +4407,13 @@
         <v>100</v>
       </c>
       <c r="AK25" t="s" s="2">
-        <v>261</v>
+        <v>244</v>
       </c>
       <c r="AL25" t="s" s="2">
-        <v>262</v>
+        <v>245</v>
       </c>
       <c r="AM25" t="s" s="2">
-        <v>263</v>
+        <v>77</v>
       </c>
       <c r="AN25" t="s" s="2">
         <v>77</v>
@@ -4240,10 +4421,10 @@
     </row>
     <row r="26" hidden="true">
       <c r="A26" t="s" s="2">
-        <v>264</v>
+        <v>246</v>
       </c>
       <c r="B26" t="s" s="2">
-        <v>264</v>
+        <v>246</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" t="s" s="2">
@@ -4266,18 +4447,20 @@
         <v>89</v>
       </c>
       <c r="K26" t="s" s="2">
-        <v>265</v>
+        <v>155</v>
       </c>
       <c r="L26" t="s" s="2">
-        <v>266</v>
+        <v>247</v>
       </c>
       <c r="M26" t="s" s="2">
-        <v>267</v>
+        <v>248</v>
       </c>
       <c r="N26" t="s" s="2">
-        <v>268</v>
-      </c>
-      <c r="O26" s="2"/>
+        <v>249</v>
+      </c>
+      <c r="O26" t="s" s="2">
+        <v>250</v>
+      </c>
       <c r="P26" t="s" s="2">
         <v>77</v>
       </c>
@@ -4325,7 +4508,7 @@
         <v>77</v>
       </c>
       <c r="AF26" t="s" s="2">
-        <v>269</v>
+        <v>251</v>
       </c>
       <c r="AG26" t="s" s="2">
         <v>78</v>
@@ -4340,10 +4523,10 @@
         <v>100</v>
       </c>
       <c r="AK26" t="s" s="2">
-        <v>226</v>
+        <v>252</v>
       </c>
       <c r="AL26" t="s" s="2">
-        <v>226</v>
+        <v>253</v>
       </c>
       <c r="AM26" t="s" s="2">
         <v>77</v>
@@ -4354,10 +4537,10 @@
     </row>
     <row r="27" hidden="true">
       <c r="A27" t="s" s="2">
-        <v>270</v>
+        <v>254</v>
       </c>
       <c r="B27" t="s" s="2">
-        <v>270</v>
+        <v>254</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" t="s" s="2">
@@ -4380,16 +4563,20 @@
         <v>89</v>
       </c>
       <c r="K27" t="s" s="2">
-        <v>165</v>
+        <v>195</v>
       </c>
       <c r="L27" t="s" s="2">
-        <v>271</v>
+        <v>255</v>
       </c>
       <c r="M27" t="s" s="2">
-        <v>272</v>
-      </c>
-      <c r="N27" s="2"/>
-      <c r="O27" s="2"/>
+        <v>256</v>
+      </c>
+      <c r="N27" t="s" s="2">
+        <v>257</v>
+      </c>
+      <c r="O27" t="s" s="2">
+        <v>258</v>
+      </c>
       <c r="P27" t="s" s="2">
         <v>77</v>
       </c>
@@ -4437,7 +4624,7 @@
         <v>77</v>
       </c>
       <c r="AF27" t="s" s="2">
-        <v>273</v>
+        <v>259</v>
       </c>
       <c r="AG27" t="s" s="2">
         <v>78</v>
@@ -4452,24 +4639,24 @@
         <v>100</v>
       </c>
       <c r="AK27" t="s" s="2">
-        <v>131</v>
+        <v>260</v>
       </c>
       <c r="AL27" t="s" s="2">
-        <v>274</v>
+        <v>261</v>
       </c>
       <c r="AM27" t="s" s="2">
-        <v>275</v>
+        <v>77</v>
       </c>
       <c r="AN27" t="s" s="2">
         <v>77</v>
       </c>
     </row>
-    <row r="28" hidden="true">
+    <row r="28">
       <c r="A28" t="s" s="2">
-        <v>276</v>
+        <v>262</v>
       </c>
       <c r="B28" t="s" s="2">
-        <v>276</v>
+        <v>262</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" t="s" s="2">
@@ -4483,26 +4670,24 @@
         <v>79</v>
       </c>
       <c r="H28" t="s" s="2">
-        <v>77</v>
+        <v>89</v>
       </c>
       <c r="I28" t="s" s="2">
         <v>77</v>
       </c>
       <c r="J28" t="s" s="2">
-        <v>77</v>
+        <v>89</v>
       </c>
       <c r="K28" t="s" s="2">
-        <v>277</v>
+        <v>184</v>
       </c>
       <c r="L28" t="s" s="2">
-        <v>278</v>
+        <v>263</v>
       </c>
       <c r="M28" t="s" s="2">
-        <v>279</v>
-      </c>
-      <c r="N28" t="s" s="2">
-        <v>280</v>
-      </c>
+        <v>264</v>
+      </c>
+      <c r="N28" s="2"/>
       <c r="O28" s="2"/>
       <c r="P28" t="s" s="2">
         <v>77</v>
@@ -4527,13 +4712,13 @@
         <v>77</v>
       </c>
       <c r="X28" t="s" s="2">
-        <v>77</v>
+        <v>112</v>
       </c>
       <c r="Y28" t="s" s="2">
-        <v>77</v>
+        <v>265</v>
       </c>
       <c r="Z28" t="s" s="2">
-        <v>77</v>
+        <v>266</v>
       </c>
       <c r="AA28" t="s" s="2">
         <v>77</v>
@@ -4551,7 +4736,7 @@
         <v>77</v>
       </c>
       <c r="AF28" t="s" s="2">
-        <v>276</v>
+        <v>262</v>
       </c>
       <c r="AG28" t="s" s="2">
         <v>78</v>
@@ -4566,13 +4751,13 @@
         <v>100</v>
       </c>
       <c r="AK28" t="s" s="2">
-        <v>77</v>
+        <v>267</v>
       </c>
       <c r="AL28" t="s" s="2">
-        <v>281</v>
+        <v>268</v>
       </c>
       <c r="AM28" t="s" s="2">
-        <v>77</v>
+        <v>269</v>
       </c>
       <c r="AN28" t="s" s="2">
         <v>77</v>
@@ -4580,10 +4765,10 @@
     </row>
     <row r="29" hidden="true">
       <c r="A29" t="s" s="2">
-        <v>282</v>
+        <v>270</v>
       </c>
       <c r="B29" t="s" s="2">
-        <v>282</v>
+        <v>270</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" t="s" s="2">
@@ -4594,7 +4779,7 @@
         <v>78</v>
       </c>
       <c r="G29" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="H29" t="s" s="2">
         <v>77</v>
@@ -4603,16 +4788,16 @@
         <v>77</v>
       </c>
       <c r="J29" t="s" s="2">
-        <v>77</v>
+        <v>89</v>
       </c>
       <c r="K29" t="s" s="2">
-        <v>222</v>
+        <v>271</v>
       </c>
       <c r="L29" t="s" s="2">
-        <v>223</v>
+        <v>272</v>
       </c>
       <c r="M29" t="s" s="2">
-        <v>224</v>
+        <v>273</v>
       </c>
       <c r="N29" s="2"/>
       <c r="O29" s="2"/>
@@ -4663,43 +4848,43 @@
         <v>77</v>
       </c>
       <c r="AF29" t="s" s="2">
-        <v>225</v>
+        <v>270</v>
       </c>
       <c r="AG29" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH29" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="AI29" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AJ29" t="s" s="2">
-        <v>77</v>
+        <v>100</v>
       </c>
       <c r="AK29" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AL29" t="s" s="2">
-        <v>226</v>
+        <v>274</v>
       </c>
       <c r="AM29" t="s" s="2">
-        <v>77</v>
+        <v>275</v>
       </c>
       <c r="AN29" t="s" s="2">
-        <v>77</v>
+        <v>276</v>
       </c>
     </row>
     <row r="30" hidden="true">
       <c r="A30" t="s" s="2">
-        <v>283</v>
+        <v>277</v>
       </c>
       <c r="B30" t="s" s="2">
-        <v>283</v>
+        <v>277</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" t="s" s="2">
-        <v>133</v>
+        <v>77</v>
       </c>
       <c r="E30" s="2"/>
       <c r="F30" t="s" s="2">
@@ -4718,17 +4903,15 @@
         <v>77</v>
       </c>
       <c r="K30" t="s" s="2">
-        <v>134</v>
+        <v>278</v>
       </c>
       <c r="L30" t="s" s="2">
-        <v>135</v>
+        <v>279</v>
       </c>
       <c r="M30" t="s" s="2">
-        <v>228</v>
-      </c>
-      <c r="N30" t="s" s="2">
-        <v>137</v>
-      </c>
+        <v>280</v>
+      </c>
+      <c r="N30" s="2"/>
       <c r="O30" s="2"/>
       <c r="P30" t="s" s="2">
         <v>77</v>
@@ -4777,7 +4960,7 @@
         <v>77</v>
       </c>
       <c r="AF30" t="s" s="2">
-        <v>232</v>
+        <v>277</v>
       </c>
       <c r="AG30" t="s" s="2">
         <v>78</v>
@@ -4789,13 +4972,13 @@
         <v>77</v>
       </c>
       <c r="AJ30" t="s" s="2">
-        <v>139</v>
+        <v>100</v>
       </c>
       <c r="AK30" t="s" s="2">
-        <v>77</v>
+        <v>281</v>
       </c>
       <c r="AL30" t="s" s="2">
-        <v>226</v>
+        <v>282</v>
       </c>
       <c r="AM30" t="s" s="2">
         <v>77</v>
@@ -4804,16 +4987,16 @@
         <v>77</v>
       </c>
     </row>
-    <row r="31" hidden="true">
+    <row r="31">
       <c r="A31" t="s" s="2">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="B31" t="s" s="2">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" t="s" s="2">
-        <v>285</v>
+        <v>77</v>
       </c>
       <c r="E31" s="2"/>
       <c r="F31" t="s" s="2">
@@ -4823,28 +5006,26 @@
         <v>79</v>
       </c>
       <c r="H31" t="s" s="2">
-        <v>77</v>
+        <v>89</v>
       </c>
       <c r="I31" t="s" s="2">
-        <v>89</v>
+        <v>77</v>
       </c>
       <c r="J31" t="s" s="2">
         <v>89</v>
       </c>
       <c r="K31" t="s" s="2">
-        <v>134</v>
+        <v>284</v>
       </c>
       <c r="L31" t="s" s="2">
+        <v>285</v>
+      </c>
+      <c r="M31" t="s" s="2">
         <v>286</v>
       </c>
-      <c r="M31" t="s" s="2">
+      <c r="N31" s="2"/>
+      <c r="O31" t="s" s="2">
         <v>287</v>
-      </c>
-      <c r="N31" t="s" s="2">
-        <v>137</v>
-      </c>
-      <c r="O31" t="s" s="2">
-        <v>143</v>
       </c>
       <c r="P31" t="s" s="2">
         <v>77</v>
@@ -4893,7 +5074,7 @@
         <v>77</v>
       </c>
       <c r="AF31" t="s" s="2">
-        <v>288</v>
+        <v>283</v>
       </c>
       <c r="AG31" t="s" s="2">
         <v>78</v>
@@ -4905,13 +5086,13 @@
         <v>77</v>
       </c>
       <c r="AJ31" t="s" s="2">
-        <v>139</v>
+        <v>100</v>
       </c>
       <c r="AK31" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AL31" t="s" s="2">
-        <v>131</v>
+        <v>288</v>
       </c>
       <c r="AM31" t="s" s="2">
         <v>77</v>
@@ -4936,7 +5117,7 @@
         <v>78</v>
       </c>
       <c r="G32" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="H32" t="s" s="2">
         <v>77</v>
@@ -4948,13 +5129,13 @@
         <v>77</v>
       </c>
       <c r="K32" t="s" s="2">
-        <v>108</v>
+        <v>195</v>
       </c>
       <c r="L32" t="s" s="2">
-        <v>290</v>
+        <v>196</v>
       </c>
       <c r="M32" t="s" s="2">
-        <v>291</v>
+        <v>197</v>
       </c>
       <c r="N32" s="2"/>
       <c r="O32" s="2"/>
@@ -4981,13 +5162,13 @@
         <v>77</v>
       </c>
       <c r="X32" t="s" s="2">
-        <v>236</v>
+        <v>77</v>
       </c>
       <c r="Y32" t="s" s="2">
-        <v>292</v>
+        <v>77</v>
       </c>
       <c r="Z32" t="s" s="2">
-        <v>293</v>
+        <v>77</v>
       </c>
       <c r="AA32" t="s" s="2">
         <v>77</v>
@@ -5005,25 +5186,25 @@
         <v>77</v>
       </c>
       <c r="AF32" t="s" s="2">
-        <v>289</v>
+        <v>198</v>
       </c>
       <c r="AG32" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH32" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="AI32" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AJ32" t="s" s="2">
-        <v>100</v>
+        <v>77</v>
       </c>
       <c r="AK32" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AL32" t="s" s="2">
-        <v>281</v>
+        <v>199</v>
       </c>
       <c r="AM32" t="s" s="2">
         <v>77</v>
@@ -5034,21 +5215,21 @@
     </row>
     <row r="33" hidden="true">
       <c r="A33" t="s" s="2">
-        <v>294</v>
+        <v>290</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>294</v>
+        <v>290</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" t="s" s="2">
-        <v>77</v>
+        <v>133</v>
       </c>
       <c r="E33" s="2"/>
       <c r="F33" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G33" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="H33" t="s" s="2">
         <v>77</v>
@@ -5060,15 +5241,17 @@
         <v>77</v>
       </c>
       <c r="K33" t="s" s="2">
-        <v>155</v>
+        <v>134</v>
       </c>
       <c r="L33" t="s" s="2">
-        <v>295</v>
+        <v>135</v>
       </c>
       <c r="M33" t="s" s="2">
-        <v>296</v>
-      </c>
-      <c r="N33" s="2"/>
+        <v>201</v>
+      </c>
+      <c r="N33" t="s" s="2">
+        <v>137</v>
+      </c>
       <c r="O33" s="2"/>
       <c r="P33" t="s" s="2">
         <v>77</v>
@@ -5105,37 +5288,37 @@
         <v>77</v>
       </c>
       <c r="AB33" t="s" s="2">
-        <v>77</v>
+        <v>202</v>
       </c>
       <c r="AC33" t="s" s="2">
-        <v>77</v>
+        <v>203</v>
       </c>
       <c r="AD33" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AE33" t="s" s="2">
-        <v>77</v>
+        <v>204</v>
       </c>
       <c r="AF33" t="s" s="2">
-        <v>294</v>
+        <v>205</v>
       </c>
       <c r="AG33" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH33" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="AI33" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AJ33" t="s" s="2">
-        <v>100</v>
+        <v>139</v>
       </c>
       <c r="AK33" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AL33" t="s" s="2">
-        <v>281</v>
+        <v>199</v>
       </c>
       <c r="AM33" t="s" s="2">
         <v>77</v>
@@ -5144,12 +5327,12 @@
         <v>77</v>
       </c>
     </row>
-    <row r="34" hidden="true">
+    <row r="34">
       <c r="A34" t="s" s="2">
-        <v>297</v>
+        <v>291</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>297</v>
+        <v>291</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" t="s" s="2">
@@ -5163,26 +5346,24 @@
         <v>88</v>
       </c>
       <c r="H34" t="s" s="2">
-        <v>77</v>
+        <v>89</v>
       </c>
       <c r="I34" t="s" s="2">
         <v>77</v>
       </c>
       <c r="J34" t="s" s="2">
-        <v>77</v>
+        <v>89</v>
       </c>
       <c r="K34" t="s" s="2">
-        <v>298</v>
+        <v>108</v>
       </c>
       <c r="L34" t="s" s="2">
-        <v>299</v>
+        <v>292</v>
       </c>
       <c r="M34" t="s" s="2">
-        <v>300</v>
-      </c>
-      <c r="N34" t="s" s="2">
-        <v>301</v>
-      </c>
+        <v>293</v>
+      </c>
+      <c r="N34" s="2"/>
       <c r="O34" s="2"/>
       <c r="P34" t="s" s="2">
         <v>77</v>
@@ -5207,13 +5388,13 @@
         <v>77</v>
       </c>
       <c r="X34" t="s" s="2">
-        <v>77</v>
+        <v>294</v>
       </c>
       <c r="Y34" t="s" s="2">
-        <v>77</v>
+        <v>295</v>
       </c>
       <c r="Z34" t="s" s="2">
-        <v>77</v>
+        <v>296</v>
       </c>
       <c r="AA34" t="s" s="2">
         <v>77</v>
@@ -5240,25 +5421,25 @@
         <v>88</v>
       </c>
       <c r="AI34" t="s" s="2">
-        <v>77</v>
+        <v>298</v>
       </c>
       <c r="AJ34" t="s" s="2">
         <v>100</v>
       </c>
       <c r="AK34" t="s" s="2">
-        <v>77</v>
+        <v>299</v>
       </c>
       <c r="AL34" t="s" s="2">
-        <v>281</v>
+        <v>300</v>
       </c>
       <c r="AM34" t="s" s="2">
-        <v>77</v>
+        <v>301</v>
       </c>
       <c r="AN34" t="s" s="2">
         <v>77</v>
       </c>
     </row>
-    <row r="35" hidden="true">
+    <row r="35">
       <c r="A35" t="s" s="2">
         <v>302</v>
       </c>
@@ -5277,16 +5458,16 @@
         <v>88</v>
       </c>
       <c r="H35" t="s" s="2">
-        <v>77</v>
+        <v>89</v>
       </c>
       <c r="I35" t="s" s="2">
         <v>77</v>
       </c>
       <c r="J35" t="s" s="2">
-        <v>77</v>
+        <v>89</v>
       </c>
       <c r="K35" t="s" s="2">
-        <v>298</v>
+        <v>195</v>
       </c>
       <c r="L35" t="s" s="2">
         <v>303</v>
@@ -5295,9 +5476,11 @@
         <v>304</v>
       </c>
       <c r="N35" t="s" s="2">
-        <v>301</v>
-      </c>
-      <c r="O35" s="2"/>
+        <v>305</v>
+      </c>
+      <c r="O35" t="s" s="2">
+        <v>306</v>
+      </c>
       <c r="P35" t="s" s="2">
         <v>77</v>
       </c>
@@ -5345,7 +5528,7 @@
         <v>77</v>
       </c>
       <c r="AF35" t="s" s="2">
-        <v>302</v>
+        <v>307</v>
       </c>
       <c r="AG35" t="s" s="2">
         <v>78</v>
@@ -5360,13 +5543,13 @@
         <v>100</v>
       </c>
       <c r="AK35" t="s" s="2">
-        <v>77</v>
+        <v>308</v>
       </c>
       <c r="AL35" t="s" s="2">
-        <v>281</v>
+        <v>309</v>
       </c>
       <c r="AM35" t="s" s="2">
-        <v>77</v>
+        <v>310</v>
       </c>
       <c r="AN35" t="s" s="2">
         <v>77</v>
@@ -5374,10 +5557,10 @@
     </row>
     <row r="36" hidden="true">
       <c r="A36" t="s" s="2">
-        <v>305</v>
+        <v>311</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>305</v>
+        <v>311</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" t="s" s="2">
@@ -5388,28 +5571,32 @@
         <v>78</v>
       </c>
       <c r="G36" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="H36" t="s" s="2">
         <v>77</v>
       </c>
       <c r="I36" t="s" s="2">
-        <v>77</v>
+        <v>89</v>
       </c>
       <c r="J36" t="s" s="2">
-        <v>77</v>
+        <v>89</v>
       </c>
       <c r="K36" t="s" s="2">
-        <v>277</v>
+        <v>108</v>
       </c>
       <c r="L36" t="s" s="2">
-        <v>306</v>
+        <v>312</v>
       </c>
       <c r="M36" t="s" s="2">
-        <v>307</v>
-      </c>
-      <c r="N36" s="2"/>
-      <c r="O36" s="2"/>
+        <v>313</v>
+      </c>
+      <c r="N36" t="s" s="2">
+        <v>314</v>
+      </c>
+      <c r="O36" t="s" s="2">
+        <v>315</v>
+      </c>
       <c r="P36" t="s" s="2">
         <v>77</v>
       </c>
@@ -5433,13 +5620,13 @@
         <v>77</v>
       </c>
       <c r="X36" t="s" s="2">
-        <v>77</v>
+        <v>294</v>
       </c>
       <c r="Y36" t="s" s="2">
-        <v>77</v>
+        <v>316</v>
       </c>
       <c r="Z36" t="s" s="2">
-        <v>77</v>
+        <v>317</v>
       </c>
       <c r="AA36" t="s" s="2">
         <v>77</v>
@@ -5457,13 +5644,13 @@
         <v>77</v>
       </c>
       <c r="AF36" t="s" s="2">
-        <v>305</v>
+        <v>318</v>
       </c>
       <c r="AG36" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH36" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="AI36" t="s" s="2">
         <v>77</v>
@@ -5472,13 +5659,13 @@
         <v>100</v>
       </c>
       <c r="AK36" t="s" s="2">
-        <v>77</v>
+        <v>319</v>
       </c>
       <c r="AL36" t="s" s="2">
-        <v>281</v>
+        <v>320</v>
       </c>
       <c r="AM36" t="s" s="2">
-        <v>77</v>
+        <v>321</v>
       </c>
       <c r="AN36" t="s" s="2">
         <v>77</v>
@@ -5486,10 +5673,10 @@
     </row>
     <row r="37" hidden="true">
       <c r="A37" t="s" s="2">
-        <v>308</v>
+        <v>322</v>
       </c>
       <c r="B37" t="s" s="2">
-        <v>308</v>
+        <v>322</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" t="s" s="2">
@@ -5509,18 +5696,20 @@
         <v>77</v>
       </c>
       <c r="J37" t="s" s="2">
-        <v>77</v>
+        <v>89</v>
       </c>
       <c r="K37" t="s" s="2">
-        <v>222</v>
+        <v>323</v>
       </c>
       <c r="L37" t="s" s="2">
-        <v>223</v>
+        <v>324</v>
       </c>
       <c r="M37" t="s" s="2">
-        <v>224</v>
-      </c>
-      <c r="N37" s="2"/>
+        <v>325</v>
+      </c>
+      <c r="N37" t="s" s="2">
+        <v>326</v>
+      </c>
       <c r="O37" s="2"/>
       <c r="P37" t="s" s="2">
         <v>77</v>
@@ -5569,7 +5758,7 @@
         <v>77</v>
       </c>
       <c r="AF37" t="s" s="2">
-        <v>225</v>
+        <v>327</v>
       </c>
       <c r="AG37" t="s" s="2">
         <v>78</v>
@@ -5581,13 +5770,13 @@
         <v>77</v>
       </c>
       <c r="AJ37" t="s" s="2">
-        <v>77</v>
+        <v>100</v>
       </c>
       <c r="AK37" t="s" s="2">
-        <v>77</v>
+        <v>199</v>
       </c>
       <c r="AL37" t="s" s="2">
-        <v>226</v>
+        <v>199</v>
       </c>
       <c r="AM37" t="s" s="2">
         <v>77</v>
@@ -5598,21 +5787,21 @@
     </row>
     <row r="38" hidden="true">
       <c r="A38" t="s" s="2">
-        <v>309</v>
+        <v>328</v>
       </c>
       <c r="B38" t="s" s="2">
-        <v>309</v>
+        <v>328</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" t="s" s="2">
-        <v>133</v>
+        <v>77</v>
       </c>
       <c r="E38" s="2"/>
       <c r="F38" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G38" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="H38" t="s" s="2">
         <v>77</v>
@@ -5621,20 +5810,18 @@
         <v>77</v>
       </c>
       <c r="J38" t="s" s="2">
-        <v>77</v>
+        <v>89</v>
       </c>
       <c r="K38" t="s" s="2">
-        <v>134</v>
+        <v>165</v>
       </c>
       <c r="L38" t="s" s="2">
-        <v>135</v>
+        <v>329</v>
       </c>
       <c r="M38" t="s" s="2">
-        <v>228</v>
-      </c>
-      <c r="N38" t="s" s="2">
-        <v>137</v>
-      </c>
+        <v>330</v>
+      </c>
+      <c r="N38" s="2"/>
       <c r="O38" s="2"/>
       <c r="P38" t="s" s="2">
         <v>77</v>
@@ -5683,28 +5870,28 @@
         <v>77</v>
       </c>
       <c r="AF38" t="s" s="2">
-        <v>232</v>
+        <v>331</v>
       </c>
       <c r="AG38" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH38" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="AI38" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AJ38" t="s" s="2">
-        <v>139</v>
+        <v>100</v>
       </c>
       <c r="AK38" t="s" s="2">
-        <v>77</v>
+        <v>131</v>
       </c>
       <c r="AL38" t="s" s="2">
-        <v>226</v>
+        <v>332</v>
       </c>
       <c r="AM38" t="s" s="2">
-        <v>77</v>
+        <v>333</v>
       </c>
       <c r="AN38" t="s" s="2">
         <v>77</v>
@@ -5712,14 +5899,14 @@
     </row>
     <row r="39" hidden="true">
       <c r="A39" t="s" s="2">
-        <v>310</v>
+        <v>334</v>
       </c>
       <c r="B39" t="s" s="2">
-        <v>310</v>
+        <v>334</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" t="s" s="2">
-        <v>285</v>
+        <v>77</v>
       </c>
       <c r="E39" s="2"/>
       <c r="F39" t="s" s="2">
@@ -5732,26 +5919,24 @@
         <v>77</v>
       </c>
       <c r="I39" t="s" s="2">
-        <v>89</v>
+        <v>77</v>
       </c>
       <c r="J39" t="s" s="2">
-        <v>89</v>
+        <v>77</v>
       </c>
       <c r="K39" t="s" s="2">
-        <v>134</v>
+        <v>335</v>
       </c>
       <c r="L39" t="s" s="2">
-        <v>286</v>
+        <v>336</v>
       </c>
       <c r="M39" t="s" s="2">
-        <v>287</v>
+        <v>337</v>
       </c>
       <c r="N39" t="s" s="2">
-        <v>137</v>
-      </c>
-      <c r="O39" t="s" s="2">
-        <v>143</v>
-      </c>
+        <v>338</v>
+      </c>
+      <c r="O39" s="2"/>
       <c r="P39" t="s" s="2">
         <v>77</v>
       </c>
@@ -5799,7 +5984,7 @@
         <v>77</v>
       </c>
       <c r="AF39" t="s" s="2">
-        <v>288</v>
+        <v>334</v>
       </c>
       <c r="AG39" t="s" s="2">
         <v>78</v>
@@ -5811,13 +5996,13 @@
         <v>77</v>
       </c>
       <c r="AJ39" t="s" s="2">
-        <v>139</v>
+        <v>100</v>
       </c>
       <c r="AK39" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AL39" t="s" s="2">
-        <v>131</v>
+        <v>339</v>
       </c>
       <c r="AM39" t="s" s="2">
         <v>77</v>
@@ -5828,10 +6013,10 @@
     </row>
     <row r="40" hidden="true">
       <c r="A40" t="s" s="2">
-        <v>311</v>
+        <v>340</v>
       </c>
       <c r="B40" t="s" s="2">
-        <v>311</v>
+        <v>340</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" t="s" s="2">
@@ -5839,7 +6024,7 @@
       </c>
       <c r="E40" s="2"/>
       <c r="F40" t="s" s="2">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="G40" t="s" s="2">
         <v>88</v>
@@ -5854,13 +6039,13 @@
         <v>77</v>
       </c>
       <c r="K40" t="s" s="2">
-        <v>222</v>
+        <v>195</v>
       </c>
       <c r="L40" t="s" s="2">
-        <v>312</v>
+        <v>196</v>
       </c>
       <c r="M40" t="s" s="2">
-        <v>313</v>
+        <v>197</v>
       </c>
       <c r="N40" s="2"/>
       <c r="O40" s="2"/>
@@ -5911,10 +6096,10 @@
         <v>77</v>
       </c>
       <c r="AF40" t="s" s="2">
-        <v>311</v>
+        <v>198</v>
       </c>
       <c r="AG40" t="s" s="2">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="AH40" t="s" s="2">
         <v>88</v>
@@ -5923,13 +6108,13 @@
         <v>77</v>
       </c>
       <c r="AJ40" t="s" s="2">
-        <v>100</v>
+        <v>77</v>
       </c>
       <c r="AK40" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AL40" t="s" s="2">
-        <v>226</v>
+        <v>199</v>
       </c>
       <c r="AM40" t="s" s="2">
         <v>77</v>
@@ -5940,21 +6125,21 @@
     </row>
     <row r="41" hidden="true">
       <c r="A41" t="s" s="2">
-        <v>314</v>
+        <v>341</v>
       </c>
       <c r="B41" t="s" s="2">
-        <v>314</v>
+        <v>341</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41" t="s" s="2">
-        <v>77</v>
+        <v>133</v>
       </c>
       <c r="E41" s="2"/>
       <c r="F41" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G41" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="H41" t="s" s="2">
         <v>77</v>
@@ -5966,15 +6151,17 @@
         <v>77</v>
       </c>
       <c r="K41" t="s" s="2">
-        <v>165</v>
+        <v>134</v>
       </c>
       <c r="L41" t="s" s="2">
-        <v>315</v>
+        <v>135</v>
       </c>
       <c r="M41" t="s" s="2">
-        <v>316</v>
-      </c>
-      <c r="N41" s="2"/>
+        <v>201</v>
+      </c>
+      <c r="N41" t="s" s="2">
+        <v>137</v>
+      </c>
       <c r="O41" s="2"/>
       <c r="P41" t="s" s="2">
         <v>77</v>
@@ -6023,25 +6210,25 @@
         <v>77</v>
       </c>
       <c r="AF41" t="s" s="2">
-        <v>314</v>
+        <v>205</v>
       </c>
       <c r="AG41" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH41" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="AI41" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AJ41" t="s" s="2">
-        <v>100</v>
+        <v>139</v>
       </c>
       <c r="AK41" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AL41" t="s" s="2">
-        <v>281</v>
+        <v>199</v>
       </c>
       <c r="AM41" t="s" s="2">
         <v>77</v>
@@ -6052,42 +6239,46 @@
     </row>
     <row r="42" hidden="true">
       <c r="A42" t="s" s="2">
-        <v>317</v>
+        <v>342</v>
       </c>
       <c r="B42" t="s" s="2">
-        <v>317</v>
+        <v>342</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42" t="s" s="2">
-        <v>77</v>
+        <v>343</v>
       </c>
       <c r="E42" s="2"/>
       <c r="F42" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G42" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="H42" t="s" s="2">
         <v>77</v>
       </c>
       <c r="I42" t="s" s="2">
-        <v>77</v>
+        <v>89</v>
       </c>
       <c r="J42" t="s" s="2">
-        <v>77</v>
+        <v>89</v>
       </c>
       <c r="K42" t="s" s="2">
-        <v>222</v>
+        <v>134</v>
       </c>
       <c r="L42" t="s" s="2">
-        <v>318</v>
+        <v>344</v>
       </c>
       <c r="M42" t="s" s="2">
-        <v>319</v>
-      </c>
-      <c r="N42" s="2"/>
-      <c r="O42" s="2"/>
+        <v>345</v>
+      </c>
+      <c r="N42" t="s" s="2">
+        <v>137</v>
+      </c>
+      <c r="O42" t="s" s="2">
+        <v>143</v>
+      </c>
       <c r="P42" t="s" s="2">
         <v>77</v>
       </c>
@@ -6135,25 +6326,25 @@
         <v>77</v>
       </c>
       <c r="AF42" t="s" s="2">
-        <v>317</v>
+        <v>346</v>
       </c>
       <c r="AG42" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH42" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="AI42" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AJ42" t="s" s="2">
-        <v>100</v>
+        <v>139</v>
       </c>
       <c r="AK42" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AL42" t="s" s="2">
-        <v>281</v>
+        <v>131</v>
       </c>
       <c r="AM42" t="s" s="2">
         <v>77</v>
@@ -6164,10 +6355,10 @@
     </row>
     <row r="43" hidden="true">
       <c r="A43" t="s" s="2">
-        <v>320</v>
+        <v>347</v>
       </c>
       <c r="B43" t="s" s="2">
-        <v>320</v>
+        <v>347</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" t="s" s="2">
@@ -6190,18 +6381,16 @@
         <v>77</v>
       </c>
       <c r="K43" t="s" s="2">
-        <v>321</v>
+        <v>108</v>
       </c>
       <c r="L43" t="s" s="2">
-        <v>322</v>
+        <v>348</v>
       </c>
       <c r="M43" t="s" s="2">
-        <v>323</v>
+        <v>349</v>
       </c>
       <c r="N43" s="2"/>
-      <c r="O43" t="s" s="2">
-        <v>324</v>
-      </c>
+      <c r="O43" s="2"/>
       <c r="P43" t="s" s="2">
         <v>77</v>
       </c>
@@ -6225,13 +6414,13 @@
         <v>77</v>
       </c>
       <c r="X43" t="s" s="2">
-        <v>77</v>
+        <v>294</v>
       </c>
       <c r="Y43" t="s" s="2">
-        <v>77</v>
+        <v>350</v>
       </c>
       <c r="Z43" t="s" s="2">
-        <v>77</v>
+        <v>351</v>
       </c>
       <c r="AA43" t="s" s="2">
         <v>77</v>
@@ -6249,7 +6438,7 @@
         <v>77</v>
       </c>
       <c r="AF43" t="s" s="2">
-        <v>320</v>
+        <v>347</v>
       </c>
       <c r="AG43" t="s" s="2">
         <v>78</v>
@@ -6267,17 +6456,1261 @@
         <v>77</v>
       </c>
       <c r="AL43" t="s" s="2">
-        <v>226</v>
+        <v>339</v>
       </c>
       <c r="AM43" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AN43" t="s" s="2">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="44" hidden="true">
+      <c r="A44" t="s" s="2">
+        <v>352</v>
+      </c>
+      <c r="B44" t="s" s="2">
+        <v>352</v>
+      </c>
+      <c r="C44" s="2"/>
+      <c r="D44" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="E44" s="2"/>
+      <c r="F44" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="G44" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="H44" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="I44" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="J44" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="K44" t="s" s="2">
+        <v>155</v>
+      </c>
+      <c r="L44" t="s" s="2">
+        <v>353</v>
+      </c>
+      <c r="M44" t="s" s="2">
+        <v>354</v>
+      </c>
+      <c r="N44" s="2"/>
+      <c r="O44" s="2"/>
+      <c r="P44" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Q44" s="2"/>
+      <c r="R44" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="S44" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="T44" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="U44" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="V44" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="W44" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="X44" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Y44" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Z44" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AA44" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AB44" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AC44" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AD44" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AE44" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AF44" t="s" s="2">
+        <v>352</v>
+      </c>
+      <c r="AG44" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH44" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="AI44" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AJ44" t="s" s="2">
+        <v>100</v>
+      </c>
+      <c r="AK44" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AL44" t="s" s="2">
+        <v>339</v>
+      </c>
+      <c r="AM44" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AN44" t="s" s="2">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="45" hidden="true">
+      <c r="A45" t="s" s="2">
+        <v>355</v>
+      </c>
+      <c r="B45" t="s" s="2">
+        <v>355</v>
+      </c>
+      <c r="C45" s="2"/>
+      <c r="D45" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="E45" s="2"/>
+      <c r="F45" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="G45" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="H45" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="I45" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="J45" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="K45" t="s" s="2">
+        <v>356</v>
+      </c>
+      <c r="L45" t="s" s="2">
+        <v>357</v>
+      </c>
+      <c r="M45" t="s" s="2">
+        <v>358</v>
+      </c>
+      <c r="N45" t="s" s="2">
+        <v>359</v>
+      </c>
+      <c r="O45" s="2"/>
+      <c r="P45" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Q45" s="2"/>
+      <c r="R45" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="S45" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="T45" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="U45" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="V45" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="W45" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="X45" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Y45" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Z45" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AA45" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AB45" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AC45" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AD45" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AE45" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AF45" t="s" s="2">
+        <v>355</v>
+      </c>
+      <c r="AG45" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH45" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="AI45" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AJ45" t="s" s="2">
+        <v>100</v>
+      </c>
+      <c r="AK45" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AL45" t="s" s="2">
+        <v>339</v>
+      </c>
+      <c r="AM45" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AN45" t="s" s="2">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="46" hidden="true">
+      <c r="A46" t="s" s="2">
+        <v>360</v>
+      </c>
+      <c r="B46" t="s" s="2">
+        <v>360</v>
+      </c>
+      <c r="C46" s="2"/>
+      <c r="D46" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="E46" s="2"/>
+      <c r="F46" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="G46" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="H46" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="I46" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="J46" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="K46" t="s" s="2">
+        <v>356</v>
+      </c>
+      <c r="L46" t="s" s="2">
+        <v>361</v>
+      </c>
+      <c r="M46" t="s" s="2">
+        <v>362</v>
+      </c>
+      <c r="N46" t="s" s="2">
+        <v>359</v>
+      </c>
+      <c r="O46" s="2"/>
+      <c r="P46" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Q46" s="2"/>
+      <c r="R46" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="S46" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="T46" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="U46" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="V46" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="W46" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="X46" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Y46" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Z46" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AA46" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AB46" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AC46" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AD46" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AE46" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AF46" t="s" s="2">
+        <v>360</v>
+      </c>
+      <c r="AG46" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH46" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="AI46" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AJ46" t="s" s="2">
+        <v>100</v>
+      </c>
+      <c r="AK46" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AL46" t="s" s="2">
+        <v>339</v>
+      </c>
+      <c r="AM46" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AN46" t="s" s="2">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="47" hidden="true">
+      <c r="A47" t="s" s="2">
+        <v>363</v>
+      </c>
+      <c r="B47" t="s" s="2">
+        <v>363</v>
+      </c>
+      <c r="C47" s="2"/>
+      <c r="D47" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="E47" s="2"/>
+      <c r="F47" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="G47" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="H47" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="I47" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="J47" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="K47" t="s" s="2">
+        <v>335</v>
+      </c>
+      <c r="L47" t="s" s="2">
+        <v>364</v>
+      </c>
+      <c r="M47" t="s" s="2">
+        <v>365</v>
+      </c>
+      <c r="N47" s="2"/>
+      <c r="O47" s="2"/>
+      <c r="P47" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Q47" s="2"/>
+      <c r="R47" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="S47" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="T47" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="U47" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="V47" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="W47" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="X47" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Y47" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Z47" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AA47" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AB47" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AC47" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AD47" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AE47" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AF47" t="s" s="2">
+        <v>363</v>
+      </c>
+      <c r="AG47" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH47" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AI47" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AJ47" t="s" s="2">
+        <v>100</v>
+      </c>
+      <c r="AK47" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AL47" t="s" s="2">
+        <v>339</v>
+      </c>
+      <c r="AM47" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AN47" t="s" s="2">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="48" hidden="true">
+      <c r="A48" t="s" s="2">
+        <v>366</v>
+      </c>
+      <c r="B48" t="s" s="2">
+        <v>366</v>
+      </c>
+      <c r="C48" s="2"/>
+      <c r="D48" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="E48" s="2"/>
+      <c r="F48" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="G48" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="H48" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="I48" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="J48" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="K48" t="s" s="2">
+        <v>195</v>
+      </c>
+      <c r="L48" t="s" s="2">
+        <v>196</v>
+      </c>
+      <c r="M48" t="s" s="2">
+        <v>197</v>
+      </c>
+      <c r="N48" s="2"/>
+      <c r="O48" s="2"/>
+      <c r="P48" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Q48" s="2"/>
+      <c r="R48" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="S48" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="T48" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="U48" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="V48" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="W48" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="X48" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Y48" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Z48" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AA48" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AB48" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AC48" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AD48" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AE48" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AF48" t="s" s="2">
+        <v>198</v>
+      </c>
+      <c r="AG48" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH48" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="AI48" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AJ48" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AK48" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AL48" t="s" s="2">
+        <v>199</v>
+      </c>
+      <c r="AM48" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AN48" t="s" s="2">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="49" hidden="true">
+      <c r="A49" t="s" s="2">
+        <v>367</v>
+      </c>
+      <c r="B49" t="s" s="2">
+        <v>367</v>
+      </c>
+      <c r="C49" s="2"/>
+      <c r="D49" t="s" s="2">
+        <v>133</v>
+      </c>
+      <c r="E49" s="2"/>
+      <c r="F49" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="G49" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="H49" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="I49" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="J49" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="K49" t="s" s="2">
+        <v>134</v>
+      </c>
+      <c r="L49" t="s" s="2">
+        <v>135</v>
+      </c>
+      <c r="M49" t="s" s="2">
+        <v>201</v>
+      </c>
+      <c r="N49" t="s" s="2">
+        <v>137</v>
+      </c>
+      <c r="O49" s="2"/>
+      <c r="P49" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Q49" s="2"/>
+      <c r="R49" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="S49" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="T49" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="U49" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="V49" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="W49" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="X49" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Y49" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Z49" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AA49" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AB49" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AC49" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AD49" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AE49" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AF49" t="s" s="2">
+        <v>205</v>
+      </c>
+      <c r="AG49" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH49" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AI49" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AJ49" t="s" s="2">
+        <v>139</v>
+      </c>
+      <c r="AK49" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AL49" t="s" s="2">
+        <v>199</v>
+      </c>
+      <c r="AM49" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AN49" t="s" s="2">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="50" hidden="true">
+      <c r="A50" t="s" s="2">
+        <v>368</v>
+      </c>
+      <c r="B50" t="s" s="2">
+        <v>368</v>
+      </c>
+      <c r="C50" s="2"/>
+      <c r="D50" t="s" s="2">
+        <v>343</v>
+      </c>
+      <c r="E50" s="2"/>
+      <c r="F50" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="G50" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="H50" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="I50" t="s" s="2">
+        <v>89</v>
+      </c>
+      <c r="J50" t="s" s="2">
+        <v>89</v>
+      </c>
+      <c r="K50" t="s" s="2">
+        <v>134</v>
+      </c>
+      <c r="L50" t="s" s="2">
+        <v>344</v>
+      </c>
+      <c r="M50" t="s" s="2">
+        <v>345</v>
+      </c>
+      <c r="N50" t="s" s="2">
+        <v>137</v>
+      </c>
+      <c r="O50" t="s" s="2">
+        <v>143</v>
+      </c>
+      <c r="P50" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Q50" s="2"/>
+      <c r="R50" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="S50" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="T50" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="U50" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="V50" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="W50" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="X50" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Y50" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Z50" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AA50" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AB50" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AC50" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AD50" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AE50" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AF50" t="s" s="2">
+        <v>346</v>
+      </c>
+      <c r="AG50" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH50" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AI50" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AJ50" t="s" s="2">
+        <v>139</v>
+      </c>
+      <c r="AK50" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AL50" t="s" s="2">
+        <v>131</v>
+      </c>
+      <c r="AM50" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AN50" t="s" s="2">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="51" hidden="true">
+      <c r="A51" t="s" s="2">
+        <v>369</v>
+      </c>
+      <c r="B51" t="s" s="2">
+        <v>369</v>
+      </c>
+      <c r="C51" s="2"/>
+      <c r="D51" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="E51" s="2"/>
+      <c r="F51" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="G51" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="H51" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="I51" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="J51" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="K51" t="s" s="2">
+        <v>195</v>
+      </c>
+      <c r="L51" t="s" s="2">
+        <v>370</v>
+      </c>
+      <c r="M51" t="s" s="2">
+        <v>371</v>
+      </c>
+      <c r="N51" s="2"/>
+      <c r="O51" s="2"/>
+      <c r="P51" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Q51" s="2"/>
+      <c r="R51" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="S51" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="T51" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="U51" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="V51" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="W51" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="X51" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Y51" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Z51" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AA51" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AB51" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AC51" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AD51" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AE51" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AF51" t="s" s="2">
+        <v>369</v>
+      </c>
+      <c r="AG51" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="AH51" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="AI51" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AJ51" t="s" s="2">
+        <v>100</v>
+      </c>
+      <c r="AK51" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AL51" t="s" s="2">
+        <v>199</v>
+      </c>
+      <c r="AM51" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AN51" t="s" s="2">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="52" hidden="true">
+      <c r="A52" t="s" s="2">
+        <v>372</v>
+      </c>
+      <c r="B52" t="s" s="2">
+        <v>372</v>
+      </c>
+      <c r="C52" s="2"/>
+      <c r="D52" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="E52" s="2"/>
+      <c r="F52" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="G52" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="H52" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="I52" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="J52" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="K52" t="s" s="2">
+        <v>165</v>
+      </c>
+      <c r="L52" t="s" s="2">
+        <v>373</v>
+      </c>
+      <c r="M52" t="s" s="2">
+        <v>374</v>
+      </c>
+      <c r="N52" s="2"/>
+      <c r="O52" s="2"/>
+      <c r="P52" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Q52" s="2"/>
+      <c r="R52" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="S52" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="T52" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="U52" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="V52" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="W52" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="X52" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Y52" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Z52" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AA52" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AB52" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AC52" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AD52" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AE52" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AF52" t="s" s="2">
+        <v>372</v>
+      </c>
+      <c r="AG52" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH52" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="AI52" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AJ52" t="s" s="2">
+        <v>100</v>
+      </c>
+      <c r="AK52" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AL52" t="s" s="2">
+        <v>339</v>
+      </c>
+      <c r="AM52" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AN52" t="s" s="2">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="53" hidden="true">
+      <c r="A53" t="s" s="2">
+        <v>375</v>
+      </c>
+      <c r="B53" t="s" s="2">
+        <v>375</v>
+      </c>
+      <c r="C53" s="2"/>
+      <c r="D53" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="E53" s="2"/>
+      <c r="F53" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="G53" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="H53" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="I53" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="J53" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="K53" t="s" s="2">
+        <v>195</v>
+      </c>
+      <c r="L53" t="s" s="2">
+        <v>376</v>
+      </c>
+      <c r="M53" t="s" s="2">
+        <v>377</v>
+      </c>
+      <c r="N53" s="2"/>
+      <c r="O53" s="2"/>
+      <c r="P53" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Q53" s="2"/>
+      <c r="R53" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="S53" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="T53" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="U53" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="V53" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="W53" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="X53" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Y53" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Z53" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AA53" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AB53" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AC53" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AD53" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AE53" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AF53" t="s" s="2">
+        <v>375</v>
+      </c>
+      <c r="AG53" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH53" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="AI53" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AJ53" t="s" s="2">
+        <v>100</v>
+      </c>
+      <c r="AK53" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AL53" t="s" s="2">
+        <v>339</v>
+      </c>
+      <c r="AM53" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AN53" t="s" s="2">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="54" hidden="true">
+      <c r="A54" t="s" s="2">
+        <v>378</v>
+      </c>
+      <c r="B54" t="s" s="2">
+        <v>378</v>
+      </c>
+      <c r="C54" s="2"/>
+      <c r="D54" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="E54" s="2"/>
+      <c r="F54" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="G54" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="H54" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="I54" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="J54" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="K54" t="s" s="2">
+        <v>379</v>
+      </c>
+      <c r="L54" t="s" s="2">
+        <v>380</v>
+      </c>
+      <c r="M54" t="s" s="2">
+        <v>381</v>
+      </c>
+      <c r="N54" s="2"/>
+      <c r="O54" t="s" s="2">
+        <v>382</v>
+      </c>
+      <c r="P54" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Q54" s="2"/>
+      <c r="R54" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="S54" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="T54" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="U54" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="V54" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="W54" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="X54" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Y54" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Z54" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AA54" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AB54" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AC54" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AD54" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AE54" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AF54" t="s" s="2">
+        <v>378</v>
+      </c>
+      <c r="AG54" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH54" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AI54" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AJ54" t="s" s="2">
+        <v>100</v>
+      </c>
+      <c r="AK54" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AL54" t="s" s="2">
+        <v>199</v>
+      </c>
+      <c r="AM54" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AN54" t="s" s="2">
         <v>77</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AN43">
+  <autoFilter ref="A1:AN54">
     <filterColumn colId="7">
       <customFilters>
         <customFilter operator="notEqual" val=" "/>
@@ -6287,7 +7720,7 @@
       <filters blank="true"/>
     </filterColumn>
   </autoFilter>
-  <conditionalFormatting sqref="A2:AI42">
+  <conditionalFormatting sqref="A2:AI53">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>$G2&lt;&gt;"Y"</formula>
     </cfRule>

</xml_diff>